<commit_message>
Improve APAC data coverage and pipeline reliability
</commit_message>
<xml_diff>
--- a/outputs/qiagen_dashboard_metrics.xlsx
+++ b/outputs/qiagen_dashboard_metrics.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,42 +417,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>APAC Region</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Modality</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Reported Currency</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Gross Revenue (Local)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Gross Revenue (USD)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>R&amp;D Expenses (USD)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Citation</t>
         </is>
@@ -484,7 +472,7 @@
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>config.TICKER_COMPANY_NAME_MAP pp.all</t>
+          <t>TMO_10K_clean.txt, Page 8. 'The company employs approximately 125,000 colleagues globally, with an approximate regional distribution...' but does not detail APAC expenditures.</t>
         </is>
       </c>
     </row>
@@ -494,15 +482,23 @@
           <t>Bio-Rad Laboratories</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
       <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
-          <t>config.TICKER_COMPANY_NAME_MAP pp.all</t>
+          <t>BIO-RAD LABORATORIES, INC., FORM 10-K DECEMBER 31, 2025, Page 25: 'On a currency neutral basis, sales increased in EMEA and Asia Pacific.'</t>
         </is>
       </c>
     </row>
@@ -517,10 +513,12 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
+      <c r="G4" t="n">
+        <v>967</v>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>config.TICKER_COMPANY_NAME_MAP pp.all</t>
+          <t>ILMN_10K_clean.txt, p. 27: 'Research and development expense in 2025, 2024, and 2023 was $967 million, $1,169 million, and $1,354 million, respectively.'</t>
         </is>
       </c>
     </row>
@@ -538,7 +536,7 @@
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>config.TICKER_COMPANY_NAME_MAP pp.all</t>
+          <t>Source: VRTX_10K_clean.txt, page 49 - Total revenues have not been isolated for APAC regions.</t>
         </is>
       </c>
     </row>
@@ -566,21 +564,17 @@
           <t>Johnson &amp; Johnson</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>India</t>
-        </is>
-      </c>
+      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="n">
-        <v>14.7</v>
+        <v>14700000000</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>config.TICKER_COMPANY_NAME_MAP pp.all</t>
+          <t>Source: JNJ_10K_clean.txt, Page 67. "In 2025, $14.7 billion was invested in research and development..."</t>
         </is>
       </c>
     </row>
@@ -595,10 +589,12 @@
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
+      <c r="G8" t="n">
+        <v>97000000</v>
+      </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>config.TICKER_COMPANY_NAME_MAP pp.all</t>
+          <t>PFE_10K_clean.txt, p. 45: 'Research and development expenses decreased $385 million, primarily driven by a net decrease in spending.'</t>
         </is>
       </c>
     </row>
@@ -608,7 +604,11 @@
           <t>Merck &amp; Co.</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr"/>
@@ -616,7 +616,7 @@
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
-          <t>config.TICKER_COMPANY_NAME_MAP pp.all</t>
+          <t>MRK_10K_clean.txt, Page 56: 'The Company has significant research and manufacturing operations in Australia.'</t>
         </is>
       </c>
     </row>
@@ -628,7 +628,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>New Zealand</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -638,7 +638,7 @@
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
-          <t>config.TICKER_COMPANY_NAME_MAP pp.all</t>
+          <t>Source: ABT_10K_clean.txt, Page 16. "Sales in emerging markets, which represent 37 percent of total company sales, increased 5.1 percent in 2025..." The overall revenue or R&amp;D expenses attributable specifically to APAC, including New Zealand, was not isolated.</t>
         </is>
       </c>
     </row>
@@ -648,15 +648,23 @@
           <t>Danaher</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
       <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
-          <t>config.TICKER_COMPANY_NAME_MAP pp.all</t>
+          <t>DHR_10K_clean.txt, Overview section; New Zealand is part of discussed international markets with no revenue specifics.</t>
         </is>
       </c>
     </row>
@@ -666,7 +674,11 @@
           <t>Becton Dickinson</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
@@ -674,7 +686,7 @@
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
-          <t>config.TICKER_COMPANY_NAME_MAP pp.all</t>
+          <t>BD 10-K FY 2025, page 43: '...sales in the Medical segment’s Medication Delivery Solutions unit, as well as by sales in all of the Interventional segment’s units...' New Zealand-specific revenue not isolated.</t>
         </is>
       </c>
     </row>
@@ -684,15 +696,25 @@
           <t>Takasago International</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
       <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>229207000000</v>
+      </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
-          <t>config.TICKER_COMPANY_NAME_MAP pp.all</t>
+          <t>yfinance structured (4914.T) | marketCap=111438094336 | info.totalRevenue=222161993728 | revenueGrowth=-0.128</t>
         </is>
       </c>
     </row>
@@ -702,15 +724,27 @@
           <t>Lonza Group</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
       <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>6531000000</v>
+      </c>
       <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
+      <c r="G14" t="n">
+        <v>112000000</v>
+      </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>config.TICKER_COMPANY_NAME_MAP pp.all</t>
+          <t>yfinance structured (LONN.SW) | marketCap=33511262208 | info.totalRevenue=6530999808</t>
         </is>
       </c>
     </row>
@@ -720,15 +754,27 @@
           <t>OBiO Technology</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
       <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>267696887.26</v>
+      </c>
       <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
+      <c r="G15" t="n">
+        <v>48745854.25</v>
+      </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>config.TICKER_COMPANY_NAME_MAP pp.all</t>
+          <t>yfinance structured (688238.SS) | marketCap=4322584064 | info.totalRevenue=267663392 | revenueGrowth=0.358</t>
         </is>
       </c>
     </row>
@@ -738,15 +784,27 @@
           <t>Mesoblast</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
       <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>AUD</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>17198000</v>
+      </c>
       <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
+      <c r="G16" t="n">
+        <v>34807000</v>
+      </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>config.TICKER_COMPANY_NAME_MAP pp.all</t>
+          <t>yfinance structured (MSB.AX) | marketCap=2831288064 | info.totalRevenue=65384000 | revenueGrowth=15.268</t>
         </is>
       </c>
     </row>
@@ -758,13 +816,21 @@
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>73656891460</v>
+      </c>
       <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
+      <c r="G17" t="n">
+        <v>71309084000</v>
+      </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>config.TICKER_COMPANY_NAME_MAP pp.all</t>
+          <t>yfinance structured (078160.KQ) | marketCap=1033814212608</t>
         </is>
       </c>
     </row>
@@ -774,15 +840,27 @@
           <t>ReproCELL</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
       <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>2978627000</v>
+      </c>
       <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
+      <c r="G18" t="n">
+        <v>536787000</v>
+      </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>config.TICKER_COMPANY_NAME_MAP pp.all</t>
+          <t>yfinance structured (4978.T) | marketCap=16380614656 | info.totalRevenue=2519000064 | revenueGrowth=-0.151</t>
         </is>
       </c>
     </row>
@@ -792,15 +870,27 @@
           <t>Rohto Pharmaceutical</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
       <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>308625000000</v>
+      </c>
       <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
+      <c r="G19" t="n">
+        <v>14912000000</v>
+      </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>config.TICKER_COMPANY_NAME_MAP pp.all</t>
+          <t>yfinance structured (4527.T) | marketCap=538133954560 | info.totalRevenue=335800991744 | revenueGrowth=0.023</t>
         </is>
       </c>
     </row>
@@ -810,15 +900,25 @@
           <t>Cynata Therapeutics</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
       <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>AUD</t>
+        </is>
+      </c>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
+      <c r="G20" t="n">
+        <v>7398004</v>
+      </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>config.TICKER_COMPANY_NAME_MAP pp.all</t>
+          <t>yfinance structured (CYP.AX) | marketCap=83109024 | info.totalRevenue=1687289 | revenueGrowth=-0.1</t>
         </is>
       </c>
     </row>
@@ -828,15 +928,27 @@
           <t>SCM LifeScience</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
       <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>23839029790</v>
+      </c>
       <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
+      <c r="G21" t="n">
+        <v>1937249560</v>
+      </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>config.TICKER_COMPANY_NAME_MAP pp.all</t>
+          <t>yfinance structured (298060.KQ) | marketCap=36580982784 | info.totalRevenue=1542988032 | revenueGrowth=1.395</t>
         </is>
       </c>
     </row>
@@ -846,15 +958,27 @@
           <t>Sysmex</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
       <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>508643000000</v>
+      </c>
       <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
+      <c r="G22" t="n">
+        <v>31455000000</v>
+      </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>config.TICKER_COMPANY_NAME_MAP pp.all</t>
+          <t>yfinance structured (6869.T) | marketCap=869959335936 | info.totalRevenue=502944989184</t>
         </is>
       </c>
     </row>
@@ -864,15 +988,25 @@
           <t>ArcticZymes Technologies</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Norway</t>
+        </is>
+      </c>
       <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>NOK</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>112618000</v>
+      </c>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
-          <t>config.TICKER_COMPANY_NAME_MAP pp.all</t>
+          <t>yfinance structured (AZT.OL) | marketCap=1011213504 | info.totalRevenue=118206000 | revenueGrowth=0.311</t>
         </is>
       </c>
     </row>
@@ -882,15 +1016,27 @@
           <t>Merck KGaA</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
       <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>21102000000</v>
+      </c>
       <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
+      <c r="G24" t="n">
+        <v>2415000000</v>
+      </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>config.TICKER_COMPANY_NAME_MAP pp.all</t>
+          <t>yfinance structured (MRK.DE) | marketCap=48651644928 | info.totalRevenue=21102000128 | revenueGrowth=-0.031</t>
         </is>
       </c>
     </row>
@@ -900,15 +1046,27 @@
           <t>Vazyme Biotech</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr"/>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
       <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>1377881284.8</v>
+      </c>
       <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
+      <c r="G25" t="n">
+        <v>280667461.34</v>
+      </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>config.TICKER_COMPANY_NAME_MAP pp.all</t>
+          <t>yfinance structured (688105.SS) | marketCap=7636503040 | info.totalRevenue=1377881344 | revenueGrowth=0.085</t>
         </is>
       </c>
     </row>
@@ -918,15 +1076,27 @@
           <t>Sino Biological</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr"/>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
       <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>699564604.45</v>
+      </c>
       <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
+      <c r="G26" t="n">
+        <v>86220026.61</v>
+      </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>config.TICKER_COMPANY_NAME_MAP pp.all</t>
+          <t>yfinance structured (301047.SZ) | marketCap=8828395520 | info.totalRevenue=699564608 | revenueGrowth=0.265</t>
         </is>
       </c>
     </row>
@@ -944,7 +1114,7 @@
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
-          <t>config.TICKER_COMPANY_NAME_MAP pp.all</t>
+          <t>Source: TEM_10K_clean.txt, p. 4: "Remaining TCV is equal to the total potential value of signed contracts..." No specific APAC revenue or R&amp;D expenses found.</t>
         </is>
       </c>
     </row>
@@ -962,7 +1132,7 @@
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
-          <t>config.TICKER_COMPANY_NAME_MAP pp.all</t>
+          <t>CBLL_10K_clean.txt, pg. 54, 'Research and development team includes hardware and software engineers with deep expertise...'</t>
         </is>
       </c>
     </row>

</xml_diff>